<commit_message>
qualidade de vida (?)
</commit_message>
<xml_diff>
--- a/Resultados/7d8_mantem3/analise.xlsx
+++ b/Resultados/7d8_mantem3/analise.xlsx
@@ -15,8 +15,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chance_acumulada" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Resumo'!$A$1:$C$35</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Distribuicao_conjunta'!$A$1:$E$65</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Resumo'!$A$1:$C$38</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Distribuicao_conjunta'!$A$1:$E$55</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Acertos'!$A$1:$C$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Desafios'!$A$1:$C$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Adaptacoes'!$A$1:$C$5</definedName>
@@ -454,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C35"/>
+  <dimension ref="A1:C38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -527,108 +527,108 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Contagem</t>
+          <t>Metodo</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Rolagens_possiveis</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="n">
-        <v>2097152</v>
+          <t>Tipo_de_analise</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Exata</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Contagem</t>
+          <t>Metodo</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Combinacoes_por_rolagem</t>
+          <t>Rolagens_teoricas</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>35</v>
+        <v>2097152</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Contagem</t>
+          <t>Metodo</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Ocorrencias_totais</t>
+          <t>Combinacoes_por_rolagem</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>73400320</v>
+        <v>35</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Verificacao</t>
+          <t>Metodo</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Soma_probabilidades_percentual</t>
+          <t>Avaliacoes_teoricas_exatas</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>100</v>
+        <v>73400320</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Acertos</t>
+          <t>Metodo</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Ocorrencias_analisadas</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>3</v>
+        <v>73400320</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Acertos</t>
+          <t>Metodo</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Mediana</t>
+          <t>Margem_erro_95_percentual</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Acertos</t>
+          <t>Verificacao</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Moda</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+          <t>Soma_probabilidades_percentual</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>100</v>
       </c>
     </row>
     <row r="12">
@@ -639,11 +639,11 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Variancia</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>1.5</v>
+        <v>2.625</v>
       </c>
     </row>
     <row r="13">
@@ -654,11 +654,11 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Desvio_padrao</t>
+          <t>Mediana</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>1.224744871391589</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14">
@@ -669,11 +669,13 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Minimo</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="n">
-        <v>0</v>
+          <t>Moda</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
     </row>
     <row r="15">
@@ -684,11 +686,11 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Primeiro_quartil</t>
+          <t>Variancia</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>2</v>
+        <v>1.078125</v>
       </c>
     </row>
     <row r="16">
@@ -699,11 +701,11 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Terceiro_quartil</t>
+          <t>Desvio_padrao</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>4</v>
+        <v>1.038327982864759</v>
       </c>
     </row>
     <row r="17">
@@ -714,37 +716,37 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Maximo</t>
+          <t>Minimo</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Desafios</t>
+          <t>Acertos</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Primeiro_quartil</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Desafios</t>
+          <t>Acertos</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Mediana</t>
+          <t>Terceiro_quartil</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
@@ -754,18 +756,16 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Desafios</t>
+          <t>Acertos</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Moda</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+          <t>Maximo</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="21">
@@ -776,11 +776,11 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Variancia</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>1.5</v>
+        <v>3.375</v>
       </c>
     </row>
     <row r="22">
@@ -791,11 +791,11 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Desvio_padrao</t>
+          <t>Mediana</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>1.224744871391589</v>
+        <v>3</v>
       </c>
     </row>
     <row r="23">
@@ -806,11 +806,13 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Minimo</t>
-        </is>
-      </c>
-      <c r="C23" s="2" t="n">
-        <v>0</v>
+          <t>Moda</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
     </row>
     <row r="24">
@@ -821,11 +823,11 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Primeiro_quartil</t>
+          <t>Variancia</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>2</v>
+        <v>1.078125</v>
       </c>
     </row>
     <row r="25">
@@ -836,11 +838,11 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Terceiro_quartil</t>
+          <t>Desvio_padrao</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>4</v>
+        <v>1.038327982864759</v>
       </c>
     </row>
     <row r="26">
@@ -851,58 +853,56 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Maximo</t>
+          <t>Minimo</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Adaptacoes</t>
+          <t>Desafios</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Primeiro_quartil</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
-        <v>1.125</v>
+        <v>3</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Adaptacoes</t>
+          <t>Desafios</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Mediana</t>
+          <t>Terceiro_quartil</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Adaptacoes</t>
+          <t>Desafios</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Moda</t>
-        </is>
-      </c>
-      <c r="C29" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+          <t>Maximo</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="30">
@@ -913,11 +913,11 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Variancia</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
-        <v>0.703125</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="31">
@@ -928,11 +928,11 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Desvio_padrao</t>
+          <t>Mediana</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
-        <v>0.8385254915624212</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32">
@@ -943,11 +943,13 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Minimo</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="n">
-        <v>0</v>
+          <t>Moda</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
       </c>
     </row>
     <row r="33">
@@ -958,11 +960,11 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Primeiro_quartil</t>
+          <t>Variancia</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
-        <v>1</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="34">
@@ -973,11 +975,11 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Terceiro_quartil</t>
+          <t>Desvio_padrao</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
-        <v>2</v>
+        <v>0.8660254037844386</v>
       </c>
     </row>
     <row r="35">
@@ -988,15 +990,60 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
+          <t>Minimo</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Adaptacoes</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Primeiro_quartil</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>Adaptacoes</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Terceiro_quartil</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>Adaptacoes</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
           <t>Maximo</t>
         </is>
       </c>
-      <c r="C35" s="2" t="n">
+      <c r="C38" s="2" t="n">
         <v>3</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C35"/>
+  <autoFilter ref="A1:C38"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1007,7 +1054,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E65"/>
+  <dimension ref="A1:E55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1157,10 +1204,10 @@
         <v>3</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>430080</v>
+        <v>860160</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>0.5859375</v>
+        <v>1.171875</v>
       </c>
     </row>
     <row r="9">
@@ -1191,10 +1238,10 @@
         <v>2</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>1290240</v>
+        <v>2150400</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>1.7578125</v>
+        <v>2.9296875</v>
       </c>
     </row>
     <row r="11">
@@ -1225,10 +1272,10 @@
         <v>1</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>1290240</v>
+        <v>1720320</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>1.7578125</v>
+        <v>2.34375</v>
       </c>
     </row>
     <row r="13">
@@ -1276,10 +1323,10 @@
         <v>2</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>1720320</v>
+        <v>1290240</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>2.34375</v>
+        <v>1.7578125</v>
       </c>
     </row>
     <row r="16">
@@ -1293,10 +1340,10 @@
         <v>3</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>860160</v>
+        <v>1720320</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>1.171875</v>
+        <v>2.34375</v>
       </c>
     </row>
     <row r="17">
@@ -1310,10 +1357,10 @@
         <v>1</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>2150400</v>
+        <v>1290240</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>2.9296875</v>
+        <v>1.7578125</v>
       </c>
     </row>
     <row r="18">
@@ -1327,10 +1374,10 @@
         <v>2</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>3010560</v>
+        <v>4730880</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>4.1015625</v>
+        <v>6.4453125</v>
       </c>
     </row>
     <row r="19">
@@ -1344,10 +1391,10 @@
         <v>3</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>430080</v>
+        <v>1720320</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>0.5859375</v>
+        <v>2.34375</v>
       </c>
     </row>
     <row r="20">
@@ -1361,10 +1408,10 @@
         <v>0</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>860160</v>
+        <v>430080</v>
       </c>
       <c r="E20" s="3" t="n">
-        <v>1.171875</v>
+        <v>0.5859375</v>
       </c>
     </row>
     <row r="21">
@@ -1378,10 +1425,10 @@
         <v>1</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>3440640</v>
+        <v>4300800</v>
       </c>
       <c r="E21" s="3" t="n">
-        <v>4.6875</v>
+        <v>5.859375</v>
       </c>
     </row>
     <row r="22">
@@ -1395,10 +1442,10 @@
         <v>2</v>
       </c>
       <c r="D22" s="2" t="n">
-        <v>1290240</v>
+        <v>3440640</v>
       </c>
       <c r="E22" s="3" t="n">
-        <v>1.7578125</v>
+        <v>4.6875</v>
       </c>
     </row>
     <row r="23">
@@ -1429,10 +1476,10 @@
         <v>1</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>1290240</v>
+        <v>2150400</v>
       </c>
       <c r="E24" s="3" t="n">
-        <v>1.7578125</v>
+        <v>2.9296875</v>
       </c>
     </row>
     <row r="25">
@@ -1480,10 +1527,10 @@
         <v>2</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>1290240</v>
+        <v>430080</v>
       </c>
       <c r="E27" s="3" t="n">
-        <v>1.7578125</v>
+        <v>0.5859375</v>
       </c>
     </row>
     <row r="28">
@@ -1497,10 +1544,10 @@
         <v>3</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>430080</v>
+        <v>860160</v>
       </c>
       <c r="E28" s="3" t="n">
-        <v>0.5859375</v>
+        <v>1.171875</v>
       </c>
     </row>
     <row r="29">
@@ -1514,10 +1561,10 @@
         <v>1</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>2150400</v>
+        <v>430080</v>
       </c>
       <c r="E29" s="3" t="n">
-        <v>2.9296875</v>
+        <v>0.5859375</v>
       </c>
     </row>
     <row r="30">
@@ -1548,10 +1595,10 @@
         <v>3</v>
       </c>
       <c r="D31" s="2" t="n">
-        <v>430080</v>
+        <v>1720320</v>
       </c>
       <c r="E31" s="3" t="n">
-        <v>0.5859375</v>
+        <v>2.34375</v>
       </c>
     </row>
     <row r="32">
@@ -1565,10 +1612,10 @@
         <v>0</v>
       </c>
       <c r="D32" s="2" t="n">
-        <v>1003520</v>
+        <v>143360</v>
       </c>
       <c r="E32" s="3" t="n">
-        <v>1.3671875</v>
+        <v>0.1953125</v>
       </c>
     </row>
     <row r="33">
@@ -1582,10 +1629,10 @@
         <v>1</v>
       </c>
       <c r="D33" s="2" t="n">
-        <v>4730880</v>
+        <v>3440640</v>
       </c>
       <c r="E33" s="3" t="n">
-        <v>6.4453125</v>
+        <v>4.6875</v>
       </c>
     </row>
     <row r="34">
@@ -1599,10 +1646,10 @@
         <v>2</v>
       </c>
       <c r="D34" s="2" t="n">
-        <v>2150400</v>
+        <v>5160960</v>
       </c>
       <c r="E34" s="3" t="n">
-        <v>2.9296875</v>
+        <v>7.03125</v>
       </c>
     </row>
     <row r="35">
@@ -1616,10 +1663,10 @@
         <v>3</v>
       </c>
       <c r="D35" s="2" t="n">
-        <v>143360</v>
+        <v>1146880</v>
       </c>
       <c r="E35" s="3" t="n">
-        <v>0.1953125</v>
+        <v>1.5625</v>
       </c>
     </row>
     <row r="36">
@@ -1633,10 +1680,10 @@
         <v>0</v>
       </c>
       <c r="D36" s="2" t="n">
-        <v>2150400</v>
+        <v>1290240</v>
       </c>
       <c r="E36" s="3" t="n">
-        <v>2.9296875</v>
+        <v>1.7578125</v>
       </c>
     </row>
     <row r="37">
@@ -1650,10 +1697,10 @@
         <v>1</v>
       </c>
       <c r="D37" s="2" t="n">
-        <v>3010560</v>
+        <v>4730880</v>
       </c>
       <c r="E37" s="3" t="n">
-        <v>4.1015625</v>
+        <v>6.4453125</v>
       </c>
     </row>
     <row r="38">
@@ -1667,10 +1714,10 @@
         <v>2</v>
       </c>
       <c r="D38" s="2" t="n">
-        <v>430080</v>
+        <v>1720320</v>
       </c>
       <c r="E38" s="3" t="n">
-        <v>0.5859375</v>
+        <v>2.34375</v>
       </c>
     </row>
     <row r="39">
@@ -1701,10 +1748,10 @@
         <v>1</v>
       </c>
       <c r="D40" s="2" t="n">
-        <v>430080</v>
+        <v>860160</v>
       </c>
       <c r="E40" s="3" t="n">
-        <v>0.5859375</v>
+        <v>1.171875</v>
       </c>
     </row>
     <row r="41">
@@ -1729,7 +1776,7 @@
         <v>4</v>
       </c>
       <c r="B42" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C42" s="2" t="n">
         <v>2</v>
@@ -1746,16 +1793,16 @@
         <v>4</v>
       </c>
       <c r="B43" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C43" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D43" s="2" t="n">
-        <v>1290240</v>
+        <v>860160</v>
       </c>
       <c r="E43" s="3" t="n">
-        <v>1.7578125</v>
+        <v>1.171875</v>
       </c>
     </row>
     <row r="44">
@@ -1763,16 +1810,16 @@
         <v>4</v>
       </c>
       <c r="B44" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C44" s="2" t="n">
         <v>2</v>
       </c>
       <c r="D44" s="2" t="n">
-        <v>1290240</v>
+        <v>1720320</v>
       </c>
       <c r="E44" s="3" t="n">
-        <v>1.7578125</v>
+        <v>2.34375</v>
       </c>
     </row>
     <row r="45">
@@ -1780,16 +1827,16 @@
         <v>4</v>
       </c>
       <c r="B45" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C45" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D45" s="2" t="n">
-        <v>860160</v>
+        <v>430080</v>
       </c>
       <c r="E45" s="3" t="n">
-        <v>1.171875</v>
+        <v>0.5859375</v>
       </c>
     </row>
     <row r="46">
@@ -1797,16 +1844,16 @@
         <v>4</v>
       </c>
       <c r="B46" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C46" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D46" s="2" t="n">
-        <v>3440640</v>
+        <v>3010560</v>
       </c>
       <c r="E46" s="3" t="n">
-        <v>4.6875</v>
+        <v>4.1015625</v>
       </c>
     </row>
     <row r="47">
@@ -1814,16 +1861,16 @@
         <v>4</v>
       </c>
       <c r="B47" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C47" s="2" t="n">
         <v>2</v>
       </c>
       <c r="D47" s="2" t="n">
-        <v>1290240</v>
+        <v>1720320</v>
       </c>
       <c r="E47" s="3" t="n">
-        <v>1.7578125</v>
+        <v>2.34375</v>
       </c>
     </row>
     <row r="48">
@@ -1831,16 +1878,16 @@
         <v>4</v>
       </c>
       <c r="B48" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C48" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D48" s="2" t="n">
-        <v>2150400</v>
+        <v>1290240</v>
       </c>
       <c r="E48" s="3" t="n">
-        <v>2.9296875</v>
+        <v>1.7578125</v>
       </c>
     </row>
     <row r="49">
@@ -1848,16 +1895,16 @@
         <v>4</v>
       </c>
       <c r="B49" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C49" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D49" s="2" t="n">
-        <v>3010560</v>
+        <v>1720320</v>
       </c>
       <c r="E49" s="3" t="n">
-        <v>4.1015625</v>
+        <v>2.34375</v>
       </c>
     </row>
     <row r="50">
@@ -1865,10 +1912,10 @@
         <v>4</v>
       </c>
       <c r="B50" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C50" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D50" s="2" t="n">
         <v>430080</v>
@@ -1879,53 +1926,53 @@
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B51" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C51" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D51" s="2" t="n">
-        <v>1720320</v>
+        <v>430080</v>
       </c>
       <c r="E51" s="3" t="n">
-        <v>2.34375</v>
+        <v>0.5859375</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B52" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C52" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D52" s="2" t="n">
-        <v>860160</v>
+        <v>430080</v>
       </c>
       <c r="E52" s="3" t="n">
-        <v>1.171875</v>
+        <v>0.5859375</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B53" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C53" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D53" s="2" t="n">
-        <v>430080</v>
+        <v>860160</v>
       </c>
       <c r="E53" s="3" t="n">
-        <v>0.5859375</v>
+        <v>1.171875</v>
       </c>
     </row>
     <row r="54">
@@ -1933,10 +1980,10 @@
         <v>5</v>
       </c>
       <c r="B54" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C54" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D54" s="2" t="n">
         <v>430080</v>
@@ -1947,193 +1994,23 @@
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B55" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C55" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D55" s="2" t="n">
-        <v>430080</v>
+        <v>143360</v>
       </c>
       <c r="E55" s="3" t="n">
-        <v>0.5859375</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="B56" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C56" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D56" s="2" t="n">
-        <v>1290240</v>
-      </c>
-      <c r="E56" s="3" t="n">
-        <v>1.7578125</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="B57" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="C57" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D57" s="2" t="n">
-        <v>1290240</v>
-      </c>
-      <c r="E57" s="3" t="n">
-        <v>1.7578125</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="B58" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="C58" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D58" s="2" t="n">
-        <v>1290240</v>
-      </c>
-      <c r="E58" s="3" t="n">
-        <v>1.7578125</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="B59" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="C59" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D59" s="2" t="n">
-        <v>1290240</v>
-      </c>
-      <c r="E59" s="3" t="n">
-        <v>1.7578125</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="B60" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="C60" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D60" s="2" t="n">
-        <v>430080</v>
-      </c>
-      <c r="E60" s="3" t="n">
-        <v>0.5859375</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="B61" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="C61" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D61" s="2" t="n">
-        <v>430080</v>
-      </c>
-      <c r="E61" s="3" t="n">
-        <v>0.5859375</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="B62" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="C62" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D62" s="2" t="n">
-        <v>143360</v>
-      </c>
-      <c r="E62" s="3" t="n">
         <v>0.1953125</v>
       </c>
     </row>
-    <row r="63">
-      <c r="A63" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="B63" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="C63" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D63" s="2" t="n">
-        <v>430080</v>
-      </c>
-      <c r="E63" s="3" t="n">
-        <v>0.5859375</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="B64" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="C64" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D64" s="2" t="n">
-        <v>430080</v>
-      </c>
-      <c r="E64" s="3" t="n">
-        <v>0.5859375</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="B65" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="C65" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D65" s="2" t="n">
-        <v>143360</v>
-      </c>
-      <c r="E65" s="3" t="n">
-        <v>0.1953125</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:E65"/>
+  <autoFilter ref="A1:E55"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2185,10 +2062,10 @@
         <v>1</v>
       </c>
       <c r="B3" s="2" t="n">
-        <v>6881280</v>
+        <v>8601600</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>9.375</v>
+        <v>11.71875</v>
       </c>
     </row>
     <row r="4">
@@ -2196,10 +2073,10 @@
         <v>2</v>
       </c>
       <c r="B4" s="2" t="n">
-        <v>17203200</v>
+        <v>23224320</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>23.4375</v>
+        <v>31.640625</v>
       </c>
     </row>
     <row r="5">
@@ -2207,10 +2084,10 @@
         <v>3</v>
       </c>
       <c r="B5" s="2" t="n">
-        <v>22937600</v>
+        <v>26521600</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>31.25</v>
+        <v>36.1328125</v>
       </c>
     </row>
     <row r="6">
@@ -2218,10 +2095,10 @@
         <v>4</v>
       </c>
       <c r="B6" s="2" t="n">
-        <v>17203200</v>
+        <v>11612160</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>23.4375</v>
+        <v>15.8203125</v>
       </c>
     </row>
     <row r="7">
@@ -2229,10 +2106,10 @@
         <v>5</v>
       </c>
       <c r="B7" s="2" t="n">
-        <v>6881280</v>
+        <v>2150400</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>9.375</v>
+        <v>2.9296875</v>
       </c>
     </row>
     <row r="8">
@@ -2240,10 +2117,10 @@
         <v>6</v>
       </c>
       <c r="B8" s="2" t="n">
-        <v>1146880</v>
+        <v>143360</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>1.5625</v>
+        <v>0.1953125</v>
       </c>
     </row>
   </sheetData>
@@ -2288,10 +2165,10 @@
         <v>0</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>1146880</v>
+        <v>143360</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>1.5625</v>
+        <v>0.1953125</v>
       </c>
     </row>
     <row r="3">
@@ -2299,10 +2176,10 @@
         <v>1</v>
       </c>
       <c r="B3" s="2" t="n">
-        <v>6881280</v>
+        <v>2150400</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>9.375</v>
+        <v>2.9296875</v>
       </c>
     </row>
     <row r="4">
@@ -2310,10 +2187,10 @@
         <v>2</v>
       </c>
       <c r="B4" s="2" t="n">
-        <v>17203200</v>
+        <v>11612160</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>23.4375</v>
+        <v>15.8203125</v>
       </c>
     </row>
     <row r="5">
@@ -2321,10 +2198,10 @@
         <v>3</v>
       </c>
       <c r="B5" s="2" t="n">
-        <v>22937600</v>
+        <v>26521600</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>31.25</v>
+        <v>36.1328125</v>
       </c>
     </row>
     <row r="6">
@@ -2332,10 +2209,10 @@
         <v>4</v>
       </c>
       <c r="B6" s="2" t="n">
-        <v>17203200</v>
+        <v>23224320</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>23.4375</v>
+        <v>31.640625</v>
       </c>
     </row>
     <row r="7">
@@ -2343,10 +2220,10 @@
         <v>5</v>
       </c>
       <c r="B7" s="2" t="n">
-        <v>6881280</v>
+        <v>8601600</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>9.375</v>
+        <v>11.71875</v>
       </c>
     </row>
     <row r="8">
@@ -2402,10 +2279,10 @@
         <v>0</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>17920000</v>
+        <v>9175040</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>24.4140625</v>
+        <v>12.5</v>
       </c>
     </row>
     <row r="3">
@@ -2413,10 +2290,10 @@
         <v>1</v>
       </c>
       <c r="B3" s="2" t="n">
-        <v>32256000</v>
+        <v>27525120</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>43.9453125</v>
+        <v>37.5</v>
       </c>
     </row>
     <row r="4">
@@ -2424,10 +2301,10 @@
         <v>2</v>
       </c>
       <c r="B4" s="2" t="n">
-        <v>19353600</v>
+        <v>27525120</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>26.3671875</v>
+        <v>37.5</v>
       </c>
     </row>
     <row r="5">
@@ -2435,10 +2312,10 @@
         <v>3</v>
       </c>
       <c r="B5" s="2" t="n">
-        <v>3870720</v>
+        <v>9175040</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>5.2734375</v>
+        <v>12.5</v>
       </c>
     </row>
   </sheetData>
@@ -2512,10 +2389,10 @@
         <v>1</v>
       </c>
       <c r="B3" s="2" t="n">
-        <v>6881280</v>
+        <v>8601600</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>9.375</v>
+        <v>11.71875</v>
       </c>
       <c r="D3" s="3" t="n">
         <v>98.4375</v>
@@ -2529,16 +2406,16 @@
         <v>2</v>
       </c>
       <c r="B4" s="2" t="n">
-        <v>17203200</v>
+        <v>23224320</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>23.4375</v>
+        <v>31.640625</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>89.0625</v>
+        <v>86.71875</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>10.9375</v>
+        <v>13.28125</v>
       </c>
     </row>
     <row r="5">
@@ -2546,16 +2423,16 @@
         <v>3</v>
       </c>
       <c r="B5" s="2" t="n">
-        <v>22937600</v>
+        <v>26521600</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>31.25</v>
+        <v>36.1328125</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>65.625</v>
+        <v>55.078125</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>34.375</v>
+        <v>44.921875</v>
       </c>
     </row>
     <row r="6">
@@ -2563,16 +2440,16 @@
         <v>4</v>
       </c>
       <c r="B6" s="2" t="n">
-        <v>17203200</v>
+        <v>11612160</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>23.4375</v>
+        <v>15.8203125</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>34.375</v>
+        <v>18.9453125</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>65.625</v>
+        <v>81.0546875</v>
       </c>
     </row>
     <row r="7">
@@ -2580,16 +2457,16 @@
         <v>5</v>
       </c>
       <c r="B7" s="2" t="n">
-        <v>6881280</v>
+        <v>2150400</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>9.375</v>
+        <v>2.9296875</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>10.9375</v>
+        <v>3.125</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>89.0625</v>
+        <v>96.875</v>
       </c>
     </row>
     <row r="8">
@@ -2597,16 +2474,16 @@
         <v>6</v>
       </c>
       <c r="B8" s="2" t="n">
-        <v>1146880</v>
+        <v>143360</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>1.5625</v>
+        <v>0.1953125</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>1.5625</v>
+        <v>0.1953125</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>98.4375</v>
+        <v>99.8046875</v>
       </c>
     </row>
   </sheetData>

</xml_diff>